<commit_message>
update to team gc
</commit_message>
<xml_diff>
--- a/LaBlanca/LaBlanca.xlsx
+++ b/LaBlanca/LaBlanca.xlsx
@@ -3663,7 +3663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3689,7 +3689,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>races</t>
+          <t>racers</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>time1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>racers1</t>
         </is>
       </c>
     </row>
@@ -3701,12 +3711,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A-P-V</t>
+          <t>WEz pb Cycling District</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01:39:19.783</t>
+          <t>31:57.682</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3715,6 +3725,14 @@
         </is>
       </c>
       <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>31:57.682</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3726,20 +3744,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>SISU Racing</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01:40:23.926</t>
+          <t>33:00.660</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>01:04.143</t>
+          <t>01:02.978</t>
         </is>
       </c>
       <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>33:00.660</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3751,146 +3777,1415 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVOLUTION </t>
+          <t>HEXAGONE.CC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>01:44:33.161</t>
+          <t>33:17.955</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05:13.378</t>
+          <t>01:20.273</t>
         </is>
       </c>
       <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>33:17.955</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>RHINO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>01:50:55.878</t>
+          <t>33:21.271</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00.000</t>
+          <t>01:23.589</t>
         </is>
       </c>
       <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>33:21.271</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RollCo</t>
+          <t>DZR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01:51:04.193</t>
+          <t>33:22.401</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08.315</t>
+          <t>01:24.719</t>
         </is>
       </c>
       <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>33:22.401</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HERC</t>
+          <t>Njinga Cycling</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>01:57:16.061</t>
+          <t>33:23.872</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06:20.183</t>
+          <t>01:26.190</t>
         </is>
       </c>
       <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>33:23.872</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>LEVEL Esports</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>01:57:37.668</t>
+          <t>33:24.482</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00.000</t>
+          <t>01:26.800</t>
         </is>
       </c>
       <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>33:24.482</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>VenTech</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>33:45.002</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>01:47.320</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>33:45.002</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>eSRT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>33:46.947</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>01:49.265</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>33:46.947</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BIKELY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>33:57.310</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>01:59.628</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>33:57.310</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DIRT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>33:57.721</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>02:00.039</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>33:57.721</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RtB</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>34:53.668</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>02:55.986</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>34:53.668</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ZSUNR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>35:38.215</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>03:40.533</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>35:38.215</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Zwift TURKIYE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>37:50.496</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>05:52.814</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>37:50.496</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>COALITION</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>01:08:53.692</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>36:56.010</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>01:08:53.692</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ATGNI</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>01:15:34.745</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>43:37.063</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>01:15:34.745</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>A-P-V</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>01:39:19.783</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>01:07:22.101</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>01:39:19.783</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Team Not Pogi</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>01:40:23.926</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>01:08:26.244</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>01:40:23.926</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EVOLUTION </t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>01:44:33.161</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>01:12:35.479</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>01:44:33.161</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Team CLS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>35:55.766</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>00.000</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>35:55.766</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DZR</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>36:22.857</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>27.091</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>36:22.857</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TZP</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>37:14.815</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>01:19.049</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>37:14.815</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HERD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>37:22.000</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>01:26.234</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>37:22.000</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>S R T</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>37:39.450</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>01:43.684</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>37:39.450</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TSE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>37:41.896</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>01:46.130</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>37:41.896</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>&amp;#128123; Ghost &amp;#128123;</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>38:05.091</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>02:09.325</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>38:05.091</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HISP</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>38:09.320</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>02:13.554</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>38:09.320</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>[GALAXY]</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>39:15.657</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>03:19.891</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>39:15.657</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RHINO</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>01:15:36.260</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>39:40.494</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>01:15:36.260</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Team Not Pogi</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>01:50:55.878</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>01:15:00.112</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>01:50:55.878</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RollCo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>01:51:04.193</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>01:15:08.427</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>01:51:04.193</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>HERC</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>01:57:16.061</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>01:21:20.295</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>01:57:16.061</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ACE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>35:10.925</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>00.000</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>35:10.925</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>S R T</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>38:04.051</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>02:53.126</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>38:04.051</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>[GALAXY]</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>38:06.428</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>02:55.503</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>38:06.428</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>38:58.416</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>03:47.491</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>38:58.416</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>39:16.112</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>04:05.187</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>39:16.112</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TBG</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>41:26.901</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>06:15.976</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>41:26.901</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CTT</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>44:34.144</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>09:23.219</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>44:34.144</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Team Not Pogi</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>01:57:37.668</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>01:22:26.743</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>01:57:37.668</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HERC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
         <is>
           <t>01:59:01.269</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>01:23.601</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>01:23:50.344</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>01:59:01.269</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Team Not Pogi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>41:36.187</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>00.000</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>41:36.187</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HERC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>45:22.447</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>03:46.260</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>45:22.447</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DBM</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>48:08.706</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>06:32.519</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>48:08.706</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>[GALAXY]</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>01:37:25.938</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>55:49.751</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>01:37:25.938</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix to team gc2
</commit_message>
<xml_diff>
--- a/LaBlanca/LaBlanca.xlsx
+++ b/LaBlanca/LaBlanca.xlsx
@@ -3711,12 +3711,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>WEz pb Cycling District</t>
+          <t>A-P-V</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>31:57.682</t>
+          <t>01:39:19.783</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3725,15 +3725,15 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>31:57.682</t>
+          <t>01:39:19.783</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -3744,29 +3744,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SISU Racing</t>
+          <t>Team Not Pogi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>33:00.660</t>
+          <t>01:40:23.926</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>01:02.978</t>
+          <t>01:04.143</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>33:00.660</t>
+          <t>01:40:23.926</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -3777,29 +3777,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HEXAGONE.CC</t>
+          <t xml:space="preserve">EVOLUTION </t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>33:17.955</t>
+          <t>01:44:33.161</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>01:20.273</t>
+          <t>05:13.378</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>33:17.955</t>
+          <t>01:44:33.161</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RHINO</t>
+          <t>COALITION</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>33:21.271</t>
+          <t>01:08:53.692</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>01:23.589</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>33:21.271</t>
+          <t>01:08:53.692</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -3843,29 +3843,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DZR</t>
+          <t>ATGNI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>33:22.401</t>
+          <t>01:15:34.745</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>01:24.719</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>33:22.401</t>
+          <t>01:15:34.745</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -3876,17 +3876,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Njinga Cycling</t>
+          <t>WEz pb Cycling District</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>33:23.872</t>
+          <t>31:57.682</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>01:26.190</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>33:23.872</t>
+          <t>31:57.682</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -3909,17 +3909,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LEVEL Esports</t>
+          <t>SISU Racing</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>33:24.482</t>
+          <t>33:00.660</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>01:26.800</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>33:24.482</t>
+          <t>33:00.660</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -3942,17 +3942,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>VenTech</t>
+          <t>HEXAGONE.CC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>33:45.002</t>
+          <t>33:17.955</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>01:47.320</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>33:45.002</t>
+          <t>33:17.955</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -3975,17 +3975,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eSRT</t>
+          <t>RHINO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>33:46.947</t>
+          <t>33:21.271</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>01:49.265</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>33:46.947</t>
+          <t>33:21.271</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -4008,17 +4008,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BIKELY</t>
+          <t>DZR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>33:57.310</t>
+          <t>33:22.401</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>01:59.628</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>33:57.310</t>
+          <t>33:22.401</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -4041,17 +4041,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DIRT</t>
+          <t>Njinga Cycling</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>33:57.721</t>
+          <t>33:23.872</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>02:00.039</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>33:57.721</t>
+          <t>33:23.872</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -4074,17 +4074,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RtB</t>
+          <t>LEVEL Esports</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>34:53.668</t>
+          <t>33:24.482</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>02:55.986</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>34:53.668</t>
+          <t>33:24.482</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -4107,17 +4107,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ZSUNR</t>
+          <t>VenTech</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>35:38.215</t>
+          <t>33:45.002</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>03:40.533</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>35:38.215</t>
+          <t>33:45.002</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -4140,17 +4140,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Zwift TURKIYE</t>
+          <t>eSRT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>37:50.496</t>
+          <t>33:46.947</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05:52.814</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>37:50.496</t>
+          <t>33:46.947</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -4173,17 +4173,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>COALITION</t>
+          <t>BIKELY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>01:08:53.692</t>
+          <t>33:57.310</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>36:56.010</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -4191,11 +4191,11 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>01:08:53.692</t>
+          <t>33:57.310</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -4206,17 +4206,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ATGNI</t>
+          <t>DIRT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>01:15:34.745</t>
+          <t>33:57.721</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>43:37.063</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -4224,11 +4224,11 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>01:15:34.745</t>
+          <t>33:57.721</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -4239,17 +4239,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>A-P-V</t>
+          <t>RtB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>01:39:19.783</t>
+          <t>34:53.668</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>01:07:22.101</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -4257,11 +4257,11 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>01:39:19.783</t>
+          <t>34:53.668</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -4272,17 +4272,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>ZSUNR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>01:40:23.926</t>
+          <t>35:38.215</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>01:08:26.244</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -4290,11 +4290,11 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>01:40:23.926</t>
+          <t>35:38.215</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -4305,17 +4305,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVOLUTION </t>
+          <t>Zwift TURKIYE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>01:44:33.161</t>
+          <t>37:50.496</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>01:12:35.479</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -4323,11 +4323,11 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>01:44:33.161</t>
+          <t>37:50.496</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -4338,12 +4338,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Team CLS</t>
+          <t>Team Not Pogi</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>35:55.766</t>
+          <t>01:50:55.878</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -4352,15 +4352,15 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>35:55.766</t>
+          <t>01:50:55.878</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -4371,29 +4371,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DZR</t>
+          <t>RollCo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>36:22.857</t>
+          <t>01:51:04.193</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>27.091</t>
+          <t>08.315</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>36:22.857</t>
+          <t>01:51:04.193</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -4404,29 +4404,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TZP</t>
+          <t>HERC</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>37:14.815</t>
+          <t>01:57:16.061</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>01:19.049</t>
+          <t>06:20.183</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>37:14.815</t>
+          <t>01:57:16.061</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -4437,29 +4437,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HERD</t>
+          <t>RHINO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>37:22.000</t>
+          <t>01:15:36.260</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>01:26.234</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>37:22.000</t>
+          <t>01:15:36.260</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -4470,17 +4470,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>S R T</t>
+          <t>Team CLS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>37:39.450</t>
+          <t>35:55.766</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>01:43.684</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>37:39.450</t>
+          <t>35:55.766</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -4503,17 +4503,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TSE</t>
+          <t>DZR</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>37:41.896</t>
+          <t>36:22.857</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>01:46.130</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>37:41.896</t>
+          <t>36:22.857</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -4536,17 +4536,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>&amp;#128123; Ghost &amp;#128123;</t>
+          <t>TZP</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>38:05.091</t>
+          <t>37:14.815</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>02:09.325</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>38:05.091</t>
+          <t>37:14.815</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -4569,17 +4569,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HISP</t>
+          <t>HERD</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>38:09.320</t>
+          <t>37:22.000</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>02:13.554</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>38:09.320</t>
+          <t>37:22.000</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -4602,17 +4602,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>[GALAXY]</t>
+          <t>S R T</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>39:15.657</t>
+          <t>37:39.450</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>03:19.891</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>39:15.657</t>
+          <t>37:39.450</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -4635,17 +4635,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RHINO</t>
+          <t>TSE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>01:15:36.260</t>
+          <t>37:41.896</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>39:40.494</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -4653,11 +4653,11 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>01:15:36.260</t>
+          <t>37:41.896</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -4668,17 +4668,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>&amp;#128123; Ghost &amp;#128123;</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>01:50:55.878</t>
+          <t>38:05.091</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>01:15:00.112</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -4686,11 +4686,11 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>01:50:55.878</t>
+          <t>38:05.091</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -4701,17 +4701,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>RollCo</t>
+          <t>HISP</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>01:51:04.193</t>
+          <t>38:09.320</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>01:15:08.427</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -4719,11 +4719,11 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>01:51:04.193</t>
+          <t>38:09.320</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -4734,17 +4734,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HERC</t>
+          <t>[GALAXY]</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>01:57:16.061</t>
+          <t>39:15.657</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>01:21:20.295</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -4752,11 +4752,11 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>01:57:16.061</t>
+          <t>39:15.657</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -4767,12 +4767,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ACE</t>
+          <t>Team Not Pogi</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>35:10.925</t>
+          <t>01:57:37.668</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4781,15 +4781,15 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>35:10.925</t>
+          <t>01:57:37.668</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -4800,29 +4800,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>S R T</t>
+          <t>HERC</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>38:04.051</t>
+          <t>01:59:01.269</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>02:53.126</t>
+          <t>01:23.601</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>38:04.051</t>
+          <t>01:59:01.269</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -4833,17 +4833,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>[GALAXY]</t>
+          <t>ACE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>38:06.428</t>
+          <t>35:10.925</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>02:55.503</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>38:06.428</t>
+          <t>35:10.925</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -4866,17 +4866,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Innovation</t>
+          <t>S R T</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>38:58.416</t>
+          <t>38:04.051</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>03:47.491</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>38:58.416</t>
+          <t>38:04.051</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -4899,17 +4899,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>[GALAXY]</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>39:16.112</t>
+          <t>38:06.428</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>04:05.187</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>39:16.112</t>
+          <t>38:06.428</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -4932,17 +4932,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TBG</t>
+          <t>Innovation</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>41:26.901</t>
+          <t>38:58.416</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>06:15.976</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>41:26.901</t>
+          <t>38:58.416</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -4965,17 +4965,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CTT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>44:34.144</t>
+          <t>39:16.112</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>09:23.219</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>44:34.144</t>
+          <t>39:16.112</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -4998,17 +4998,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>TBG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>01:57:37.668</t>
+          <t>41:26.901</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>01:22:26.743</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -5016,11 +5016,11 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01:57:37.668</t>
+          <t>41:26.901</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -5031,17 +5031,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>HERC</t>
+          <t>CTT</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>01:59:01.269</t>
+          <t>44:34.144</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>01:23:50.344</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -5049,11 +5049,11 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>01:59:01.269</t>
+          <t>44:34.144</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -5064,12 +5064,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>[GALAXY]</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>41:36.187</t>
+          <t>01:37:25.938</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5078,15 +5078,15 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>41:36.187</t>
+          <t>01:37:25.938</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -5097,17 +5097,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>HERC</t>
+          <t>Team Not Pogi</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>45:22.447</t>
+          <t>41:36.187</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>03:46.260</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>45:22.447</t>
+          <t>41:36.187</t>
         </is>
       </c>
       <c r="G44" t="n">
@@ -5130,17 +5130,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DBM</t>
+          <t>HERC</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>48:08.706</t>
+          <t>45:22.447</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>06:32.519</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>48:08.706</t>
+          <t>45:22.447</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -5163,17 +5163,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>[GALAXY]</t>
+          <t>DBM</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>01:37:25.938</t>
+          <t>48:08.706</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>55:49.751</t>
+          <t>00.000</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5181,11 +5181,11 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01:37:25.938</t>
+          <t>48:08.706</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>